<commit_message>
Update integration tests and replace request package.
Ticket: https://github.com/SiLeBAT/mibi-portal-server/issues/463
Ticket: https://github.com/SiLeBAT/mibi-portal-server/issues/287
</commit_message>
<xml_diff>
--- a/test/data/mps155_timezone_bug_v17.xlsx
+++ b/test/data/mps155_timezone_bug_v17.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="184">
   <si>
     <r>
       <rPr>
@@ -443,6 +443,9 @@
   </si>
   <si>
     <t xml:space="preserve">Email-Adresse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test@test.de</t>
   </si>
   <si>
     <r>
@@ -3094,9 +3097,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>773280</xdr:colOff>
+      <xdr:colOff>772920</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>282960</xdr:rowOff>
+      <xdr:rowOff>282600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3109,8 +3112,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11756520" y="38160"/>
-          <a:ext cx="1613880" cy="673200"/>
+          <a:off x="11754720" y="38160"/>
+          <a:ext cx="1613160" cy="672840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3137,7 +3140,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="10.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="10.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10.29"/>
@@ -3702,7 +3705,9 @@
         <v>41</v>
       </c>
       <c r="B22" s="29"/>
-      <c r="C22" s="25"/>
+      <c r="C22" s="25" t="s">
+        <v>42</v>
+      </c>
       <c r="D22" s="25"/>
       <c r="E22" s="25"/>
       <c r="F22" s="25"/>
@@ -3710,7 +3715,7 @@
       <c r="H22" s="25"/>
       <c r="I22" s="26"/>
       <c r="J22" s="28" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K22" s="28"/>
       <c r="L22" s="28"/>
@@ -3722,7 +3727,7 @@
       <c r="R22" s="23"/>
       <c r="S22" s="23"/>
       <c r="W22" s="30" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" s="6" customFormat="true" ht="17.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3820,7 +3825,7 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
       <c r="J27" s="37" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K27" s="5"/>
       <c r="L27" s="29" t="s">
@@ -3836,7 +3841,7 @@
     </row>
     <row r="28" s="6" customFormat="true" ht="17.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="38" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B28" s="38"/>
       <c r="C28" s="4"/>
@@ -3880,7 +3885,7 @@
     </row>
     <row r="30" s="6" customFormat="true" ht="17.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="42" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B30" s="42"/>
       <c r="C30" s="42"/>
@@ -3903,7 +3908,7 @@
     </row>
     <row r="31" s="6" customFormat="true" ht="17.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="44" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B31" s="44"/>
       <c r="C31" s="44"/>
@@ -3947,7 +3952,7 @@
     </row>
     <row r="33" s="46" customFormat="true" ht="17.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="47" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B33" s="47"/>
       <c r="C33" s="48"/>
@@ -4012,7 +4017,7 @@
     </row>
     <row r="36" s="46" customFormat="true" ht="17.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="50" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B36" s="50"/>
       <c r="C36" s="50"/>
@@ -4035,7 +4040,7 @@
     </row>
     <row r="37" s="6" customFormat="true" ht="17.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="40" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B37" s="40"/>
       <c r="C37" s="40"/>
@@ -4058,7 +4063,7 @@
     </row>
     <row r="38" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="51" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B38" s="51"/>
       <c r="C38" s="51"/>
@@ -4134,82 +4139,82 @@
     </row>
     <row r="41" s="56" customFormat="true" ht="109.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="63" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B41" s="64" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C41" s="65" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D41" s="63" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E41" s="65" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F41" s="63" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G41" s="65" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H41" s="63" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I41" s="66" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J41" s="65" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K41" s="63" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L41" s="66" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M41" s="67" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N41" s="65" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O41" s="63" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P41" s="66" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q41" s="65" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R41" s="63" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="S41" s="65" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="T41" s="68" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="U41" s="68" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="V41" s="68" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" s="78" customFormat="true" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="69" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B42" s="70" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C42" s="71"/>
       <c r="D42" s="72" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E42" s="71"/>
       <c r="F42" s="73" t="n">
@@ -4219,40 +4224,40 @@
         <v>43467</v>
       </c>
       <c r="H42" s="75" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I42" s="76" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J42" s="71" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K42" s="69" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L42" s="76" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M42" s="75" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N42" s="71" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O42" s="69" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="P42" s="76" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q42" s="71" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="R42" s="69" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="S42" s="71" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="T42" s="77"/>
       <c r="U42" s="77"/>
@@ -4260,14 +4265,14 @@
     </row>
     <row r="43" s="86" customFormat="true" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="69" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B43" s="79" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C43" s="80"/>
       <c r="D43" s="75" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E43" s="71"/>
       <c r="F43" s="81" t="n">
@@ -4277,40 +4282,40 @@
         <v>43466</v>
       </c>
       <c r="H43" s="75" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I43" s="76" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J43" s="71" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K43" s="83" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L43" s="84" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M43" s="75" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="N43" s="71" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O43" s="69" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="P43" s="76" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q43" s="71" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="R43" s="83" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S43" s="75" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="T43" s="85"/>
       <c r="U43" s="77"/>
@@ -30425,7 +30430,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="125" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B1" s="126"/>
       <c r="C1" s="126"/>
@@ -30483,7 +30488,7 @@
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="129" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B3" s="130"/>
       <c r="C3" s="130"/>
@@ -30513,19 +30518,19 @@
     </row>
     <row r="4" customFormat="false" ht="39" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="132" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B4" s="133" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C4" s="134" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D4" s="135" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E4" s="136" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F4" s="137"/>
       <c r="G4" s="128"/>
@@ -30551,19 +30556,19 @@
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="138" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B5" s="139" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C5" s="140" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D5" s="141" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E5" s="142" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F5" s="137"/>
       <c r="G5" s="128"/>
@@ -30589,17 +30594,17 @@
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="143" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B6" s="144" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C6" s="145" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D6" s="146"/>
       <c r="E6" s="147" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F6" s="137"/>
       <c r="G6" s="128"/>
@@ -30625,17 +30630,17 @@
     </row>
     <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="148" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B7" s="149" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C7" s="150" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D7" s="151"/>
       <c r="E7" s="152" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F7" s="137"/>
       <c r="G7" s="128"/>
@@ -30661,19 +30666,19 @@
     </row>
     <row r="8" customFormat="false" ht="76.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="138" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B8" s="139" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C8" s="140" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D8" s="141" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E8" s="142" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F8" s="137"/>
       <c r="G8" s="128"/>
@@ -30699,13 +30704,13 @@
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="148" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B9" s="149" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C9" s="153" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D9" s="154"/>
       <c r="E9" s="152"/>
@@ -30733,19 +30738,19 @@
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="138" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B10" s="139" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C10" s="140" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D10" s="141" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E10" s="142" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F10" s="137"/>
       <c r="G10" s="128"/>
@@ -30771,17 +30776,17 @@
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="148" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B11" s="149" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" s="153" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D11" s="154"/>
       <c r="E11" s="152" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F11" s="137"/>
       <c r="G11" s="128"/>
@@ -30807,17 +30812,17 @@
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="138" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B12" s="139" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C12" s="140" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D12" s="135"/>
       <c r="E12" s="136" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F12" s="137"/>
       <c r="G12" s="128"/>
@@ -30843,13 +30848,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="143" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B13" s="144" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C13" s="145" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D13" s="135"/>
       <c r="E13" s="136"/>
@@ -30877,13 +30882,13 @@
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="148" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B14" s="149" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C14" s="153" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D14" s="135"/>
       <c r="E14" s="136"/>
@@ -30911,19 +30916,19 @@
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="138" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B15" s="139" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C15" s="140" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D15" s="141" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E15" s="142" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F15" s="137"/>
       <c r="G15" s="128"/>
@@ -30949,13 +30954,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="143" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B16" s="144" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C16" s="145" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D16" s="141"/>
       <c r="E16" s="142"/>
@@ -30983,13 +30988,13 @@
     </row>
     <row r="17" customFormat="false" ht="63.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="143" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B17" s="144" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C17" s="145" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D17" s="141"/>
       <c r="E17" s="142"/>
@@ -31017,13 +31022,13 @@
     </row>
     <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="148" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B18" s="149" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C18" s="153" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D18" s="154"/>
       <c r="E18" s="152"/>
@@ -31051,17 +31056,17 @@
     </row>
     <row r="19" customFormat="false" ht="38.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="138" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B19" s="139" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C19" s="140" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D19" s="141"/>
       <c r="E19" s="142" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F19" s="137"/>
       <c r="G19" s="128"/>
@@ -31087,13 +31092,13 @@
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="143" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B20" s="144" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C20" s="145" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D20" s="146"/>
       <c r="E20" s="147"/>
@@ -31121,17 +31126,17 @@
     </row>
     <row r="21" customFormat="false" ht="39" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="148" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B21" s="149" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C21" s="153" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D21" s="154"/>
       <c r="E21" s="155" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F21" s="137"/>
       <c r="G21" s="128"/>
@@ -31157,13 +31162,13 @@
     </row>
     <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="138" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B22" s="139" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C22" s="140" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D22" s="141"/>
       <c r="E22" s="142"/>
@@ -31191,17 +31196,17 @@
     </row>
     <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="148" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B23" s="149" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C23" s="153" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D23" s="154"/>
       <c r="E23" s="152" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F23" s="137"/>
       <c r="G23" s="128"/>
@@ -31227,13 +31232,13 @@
     </row>
     <row r="24" s="164" customFormat="true" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="156" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B24" s="157" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C24" s="158" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D24" s="159"/>
       <c r="E24" s="160"/>
@@ -31261,17 +31266,17 @@
     </row>
     <row r="25" s="164" customFormat="true" ht="25.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="165" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B25" s="166" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" s="167" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D25" s="168"/>
       <c r="E25" s="169" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F25" s="161"/>
       <c r="G25" s="162"/>
@@ -31297,13 +31302,13 @@
     </row>
     <row r="26" s="164" customFormat="true" ht="51.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="148" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B26" s="149" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C26" s="170" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D26" s="171"/>
       <c r="E26" s="172"/>
@@ -31359,7 +31364,7 @@
     </row>
     <row r="28" s="164" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="175" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B28" s="162"/>
       <c r="C28" s="162"/>
@@ -31389,7 +31394,7 @@
     </row>
     <row r="29" s="179" customFormat="true" ht="51.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="177" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B29" s="177"/>
       <c r="C29" s="177"/>
@@ -31447,7 +31452,7 @@
     </row>
     <row r="31" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="181" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B31" s="181"/>
       <c r="C31" s="181"/>
@@ -31504,7 +31509,7 @@
     </row>
     <row r="33" s="187" customFormat="true" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="188" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B33" s="188"/>
       <c r="C33" s="188"/>
@@ -31562,7 +31567,7 @@
     </row>
     <row r="35" s="187" customFormat="true" ht="51.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="190" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B35" s="190"/>
       <c r="C35" s="190"/>
@@ -31592,7 +31597,7 @@
     </row>
     <row r="36" s="187" customFormat="true" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="191" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B36" s="191"/>
       <c r="C36" s="191"/>
@@ -31622,7 +31627,7 @@
     </row>
     <row r="37" s="187" customFormat="true" ht="12.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="191" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B37" s="191"/>
       <c r="C37" s="191"/>
@@ -31652,7 +31657,7 @@
     </row>
     <row r="38" s="187" customFormat="true" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="191" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B38" s="191"/>
       <c r="C38" s="191"/>
@@ -31682,7 +31687,7 @@
     </row>
     <row r="39" s="187" customFormat="true" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="191" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B39" s="191"/>
       <c r="C39" s="191"/>
@@ -31712,7 +31717,7 @@
     </row>
     <row r="40" s="187" customFormat="true" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="191" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B40" s="191"/>
       <c r="C40" s="191"/>
@@ -31742,7 +31747,7 @@
     </row>
     <row r="41" s="187" customFormat="true" ht="12.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="188" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B41" s="188"/>
       <c r="C41" s="188"/>

</xml_diff>